<commit_message>
feat: update project list to reference xlsx file correctly
</commit_message>
<xml_diff>
--- a/reference/us_reconductoring_projects.xlsx
+++ b/reference/us_reconductoring_projects.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marck\Documents\New project\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76CC4CBB-24C7-4A7C-8B59-9CC7F3FE8E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672FCAC0-4584-4E37-9D16-71BC93DE7079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="230" windowWidth="37560" windowHeight="20630" xr2:uid="{523144C7-1C9B-4B11-AC55-770246128A53}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="36110" windowHeight="19510" activeTab="1" xr2:uid="{523144C7-1C9B-4B11-AC55-770246128A53}"/>
   </bookViews>
   <sheets>
     <sheet name="CAISO" sheetId="1" r:id="rId1"/>
-    <sheet name="ISO-NE" sheetId="3" r:id="rId2"/>
-    <sheet name="NYISO" sheetId="4" r:id="rId3"/>
-    <sheet name="ERCOT" sheetId="5" r:id="rId4"/>
-    <sheet name="SPP" sheetId="6" r:id="rId5"/>
-    <sheet name="PJM" sheetId="7" r:id="rId6"/>
+    <sheet name="PJM" sheetId="7" r:id="rId2"/>
+    <sheet name="ISO-NE" sheetId="3" r:id="rId3"/>
+    <sheet name="NYISO" sheetId="4" r:id="rId4"/>
+    <sheet name="ERCOT" sheetId="5" r:id="rId5"/>
+    <sheet name="SPP" sheetId="6" r:id="rId6"/>
     <sheet name="MISO" sheetId="2" r:id="rId7"/>
     <sheet name="WestConnect" sheetId="8" r:id="rId8"/>
     <sheet name="NorthernGrid" sheetId="9" r:id="rId9"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="172">
   <si>
     <t>JULIAN HINDS</t>
   </si>
@@ -349,9 +349,6 @@
     <t>116 - 232</t>
   </si>
   <si>
-    <t>1350 A</t>
-  </si>
-  <si>
     <t>To mitigate P1 overloads identified as part of Interconnection Alternative E, the ISO is recommending approval. It will  take an estimated 24 months to complete.</t>
   </si>
   <si>
@@ -377,19 +374,214 @@
   </si>
   <si>
     <t>Lugo - Victor-Kramer Upgrade (3/3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warnerville-Bellota 230 kV line reconductoring </t>
+  </si>
+  <si>
+    <t>WARNERVILLE</t>
+  </si>
+  <si>
+    <t>BELLOTA</t>
+  </si>
+  <si>
+    <t>Capacity</t>
+  </si>
+  <si>
+    <t>1890 A</t>
+  </si>
+  <si>
+    <t>In Operation</t>
+  </si>
+  <si>
+    <t>The project proposes to reinforce 45 circuit miles of the 230 kV transmission lines between Bellota, Cottle, and Warnerville substations with 1113 kcmil steel-supported aluminum conductors with emergency capability of 1890 Amps. The project includes the installation of a new Optical Ground Wire (OPGW) that will replace the existing aging third-party owned OPGW.</t>
+  </si>
+  <si>
+    <t>MIDWAY</t>
+  </si>
+  <si>
+    <t>KERN</t>
+  </si>
+  <si>
+    <t>Midway – Kern PP 230 kV Line (Bakersfield-Kern Reconductor)</t>
+  </si>
+  <si>
+    <t>PG&amp;E proposes to raise approximately half of the existing towers along the line (approximately 60) approximately 7 to 27 feet by adding new extensions to the towers. Minor foundation upgrades and one foundation replacement will be completed on these towers as needed. The tower raises are required to support the new conductors, meet current design standards, reduce electric and magnetic fields near residences, and comply with minimum ground-to-conductor clearance requirements.</t>
+  </si>
+  <si>
+    <t>Q1-2024: This project is part of a multi-phased process to rebuild/reconductor in the Ripon-Manteca area. Long lead materials expected in Q1 2026. Permit completion is expected in Q1 2026. Project is soliciting bids for the design contract. Reconductor Ripon-Manteca 115 kV line 1.51 mi section of 2/0 CU and 0.92 mi 4/0 ACSR (2.43 mi total)</t>
+  </si>
+  <si>
+    <t>MANTECA</t>
+  </si>
+  <si>
+    <t>RIPON</t>
+  </si>
+  <si>
+    <t>6.8 - 13.6</t>
+  </si>
+  <si>
+    <t>Ripon-Riverbank 115 kV Line Reconductor</t>
+  </si>
+  <si>
+    <t>RIVERBANK</t>
+  </si>
+  <si>
+    <t>Manteca-Ripon 115 kV Line Reconductor</t>
+  </si>
+  <si>
+    <t>MELONES</t>
+  </si>
+  <si>
+    <t>Riverbank-Melones 115 kV Line Reconductor</t>
+  </si>
+  <si>
+    <t>Midway-Temblor 115 kV Line Reconductor and Voltage Support</t>
+  </si>
+  <si>
+    <t>TEMBLOR</t>
+  </si>
+  <si>
+    <t>Herndon-Bullard 115 kV Reconductoring Project</t>
+  </si>
+  <si>
+    <t>HERNDON</t>
+  </si>
+  <si>
+    <t>BULLARD</t>
+  </si>
+  <si>
+    <t>Category P2 overloads identified on sections of the Herndon-Bullard # 1 &amp; # 2 lines. The P2 overloads are due to loss of either of the two parallel circuits from Herndon to Pinedale Junction resulting in one of the feeds serving the entire load at Bullard and Pinedale substation.</t>
+  </si>
+  <si>
+    <t>In Flight</t>
+  </si>
+  <si>
+    <t>Christie-Sobrante 115 kV Line Reconductor</t>
+  </si>
+  <si>
+    <t>Reconductor the Christie - Sobrante 115 kV line with a larger capacity conductor</t>
+  </si>
+  <si>
+    <t>1228 MW</t>
+  </si>
+  <si>
+    <t>6 - 8</t>
+  </si>
+  <si>
+    <t>1300 A / 188 MW</t>
+  </si>
+  <si>
+    <t>1350 A / 706 MW</t>
+  </si>
+  <si>
+    <t>124 MW</t>
+  </si>
+  <si>
+    <t>CHRISTIE</t>
+  </si>
+  <si>
+    <t>SOBRANTE</t>
+  </si>
+  <si>
+    <t>Borden-Storey 230 kV 1 and 2 Line Reconductoring</t>
+  </si>
+  <si>
+    <t>1287 MW</t>
+  </si>
+  <si>
+    <t>Initiating</t>
+  </si>
+  <si>
+    <t>BORDEN CO</t>
+  </si>
+  <si>
+    <t>STORY</t>
+  </si>
+  <si>
+    <t>RAS was considered as an alternative but was not selected due to not meeting the RAS guiedlines. Series compensation was also considered as an alternative but was not selected due to the size that would be needed to mitigate the overload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wilson-Le Grand 115 kV line reconductoring </t>
+  </si>
+  <si>
+    <t>LE GRAND</t>
+  </si>
+  <si>
+    <t>Following a re-scope of the project to replace aging conductors with upgraded lines. It aims to support regional reliability and manage increasing electrical demand in Merced County, California.</t>
+  </si>
+  <si>
+    <t>MORAGA</t>
+  </si>
+  <si>
+    <t>OAKLAND X</t>
+  </si>
+  <si>
+    <t>2288 A</t>
+  </si>
+  <si>
+    <t>125 - 250</t>
+  </si>
+  <si>
+    <t>This project aims to provide a comprehensive solution to address the high demand growth in South Oakland by upgrading five 115 kV lines which serve as the primary source in this pocket. By increasing transmission capacity for serving South Oakland Pocket, this project will ensure long-term reliability of the grid and its ability to serve the growing needs.</t>
+  </si>
+  <si>
+    <t>SAN LEANDRO U</t>
+  </si>
+  <si>
+    <t>South Oakland Reinforcement Project 1</t>
+  </si>
+  <si>
+    <t>South Oakland Reinforcement Project 2</t>
+  </si>
+  <si>
+    <t>South Oakland Reinforcement Project 3</t>
+  </si>
+  <si>
+    <t>Gold Hill-El Dorado Reinforcement Project</t>
+  </si>
+  <si>
+    <t>63.5 - 127</t>
+  </si>
+  <si>
+    <t>This is just a part of the whole reinforcement project to reconductor approximately 8.8 circuit miles between El Dorado and 008/062 of the El Dorado – Missouri Flat #2 115 kV Line with larger conductor to achieve minimum 577 Amps of summer emergency rating; and</t>
+  </si>
+  <si>
+    <t>577 A</t>
+  </si>
+  <si>
+    <t>EL DORADO</t>
+  </si>
+  <si>
+    <t>MISSOURI CITY</t>
+  </si>
+  <si>
+    <t>Reconductor ES's section of the 381 (Vernon - Northfield) 345 kV line. (NH portion)</t>
+  </si>
+  <si>
+    <t>VERNON VT</t>
+  </si>
+  <si>
+    <t>NORTHFIELD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -400,7 +592,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -408,11 +600,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -423,7 +630,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -760,10 +973,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EC2192C-A7CA-4BFB-9C7D-B34D8285D403}">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="48.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.453125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.36328125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.54296875" style="2" bestFit="1" customWidth="1"/>
@@ -772,7 +985,7 @@
     <col min="7" max="7" width="11.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.26953125" style="2" customWidth="1"/>
     <col min="9" max="9" width="9.7265625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="7.36328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.36328125" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="95.81640625" style="2" customWidth="1"/>
     <col min="13" max="16384" width="10.90625" style="2"/>
@@ -782,7 +995,7 @@
       <c r="A1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -1333,7 +1546,7 @@
         <v>26</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>41</v>
+        <v>142</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>79</v>
@@ -1459,12 +1672,12 @@
         <v>2028</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>98</v>
@@ -1485,7 +1698,7 @@
         <v>41</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>99</v>
@@ -1497,18 +1710,18 @@
         <v>2034</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>105</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>72</v>
@@ -1517,16 +1730,16 @@
         <v>41</v>
       </c>
       <c r="F20" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>10</v>
@@ -1535,11 +1748,544 @@
         <v>2033</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="58" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F21" s="2">
+        <v>230</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I21" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K21" s="2">
+        <v>2024</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F22" s="2">
+        <v>230</v>
+      </c>
+      <c r="G22" s="2">
+        <v>21</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="K22" s="5">
+        <v>2025</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F23" s="2">
+        <v>115</v>
+      </c>
+      <c r="G23" s="2">
+        <v>2.4</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="K23" s="2">
+        <v>2029</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F24" s="2">
+        <v>115</v>
+      </c>
+      <c r="G24" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="K24" s="2">
+        <v>2029</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F25" s="2">
+        <v>115</v>
+      </c>
+      <c r="G25" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="K25" s="2">
+        <v>2029</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F26" s="2">
+        <v>115</v>
+      </c>
+      <c r="G26" s="2">
+        <v>15</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K26" s="2">
+        <v>2030</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F27" s="2">
+        <v>115</v>
+      </c>
+      <c r="G27" s="2">
+        <v>8</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K27" s="2">
+        <v>2028</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F28" s="2">
+        <v>115</v>
+      </c>
+      <c r="G28" s="2">
+        <v>13</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K28" s="2">
+        <v>2029</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F29" s="2">
+        <v>230</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="I29" s="2">
+        <v>74</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="K29" s="2">
+        <v>2029</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F30" s="2">
+        <v>115</v>
+      </c>
+      <c r="G30" s="2">
+        <v>3.2</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K30" s="2">
+        <v>2023</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="58" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F31" s="2">
+        <v>115</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K31" s="2">
+        <v>2032</v>
+      </c>
+      <c r="L31" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="58" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F32" s="2">
+        <v>115</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K32" s="2">
+        <v>2032</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="58" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F33" s="2">
+        <v>115</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K33" s="2">
+        <v>2032</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F34" s="2">
+        <v>115</v>
+      </c>
+      <c r="G34" s="2">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K34" s="2">
+        <v>2032</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1562,15 +2308,118 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65E6E5BD-FED4-4A95-AA13-A8D851AB1156}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9DF5F0D-5165-4A07-85C6-A5D3E3727E91}">
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65E6E5BD-FED4-4A95-AA13-A8D851AB1156}">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="67" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C5EAB86-F637-4E0B-B868-90A9F4839B36}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1579,7 +2428,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50132E97-E219-41C2-95B3-622798551570}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1588,17 +2437,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B22ADC3-2FDF-4632-9C47-C11A802298C0}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9DF5F0D-5165-4A07-85C6-A5D3E3727E91}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>

</xml_diff>